<commit_message>
dummy data changed 10:29AM
</commit_message>
<xml_diff>
--- a/Dummy Data 1.xlsx
+++ b/Dummy Data 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Balasurya Sivakumar\Desktop\dummy project for github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC62461-EE7C-4997-A110-98D33F489FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9A0F2A-FF85-4516-B939-33C87BE93E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,9 +25,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>dummy data</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>S.No</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
 </sst>
 </file>
@@ -345,12 +363,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="B2:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
         <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>